<commit_message>
Simple Flow V2 RECONCILIATION: spec v21->v23 + tech plan + designs folded in
Designs byte-identical to authoring baseline. Tech plan (new, was MISSING) confirms the suite; API
endpoints corroborate (no new cases; Rule 4 not triggered). Spec moved v21->v23 — only Story 7 changed:
SFV2-BULK-02 updated (Create invoice removed from the More ordered list). All 61 cases re-pinned to v23
(re-verified). SFV2-MENU-01 gains a disclosed divergence (tech plan: service WOs block Uncomplete at
'complete' vs spec invoiced/paid) -> PO-SF-3. Import regenerated (61 rows); coverage 21/21; RUA unaffected.
Lock released. No TestRail/Jira writes.
</commit_message>
<xml_diff>
--- a/build/simple-flow-v2/questions-2026-08-21/Questions-for-Milos-Vasic_Simple-Flow-V2_2026-08-21.xlsx
+++ b/build/simple-flow-v2/questions-2026-08-21/Questions-for-Milos-Vasic_Simple-Flow-V2_2026-08-21.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Questions - Simple Flow V2" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="QA internal - not for Milos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="QA internal" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -430,21 +430,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="56" customWidth="1" min="3" max="3"/>
-    <col width="58" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="58" customWidth="1" min="3" max="3"/>
+    <col width="56" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Questions - Simple Flow V2 - Milos Vasic - 2026-08-21</t>
+          <t>Questions - Simple Flow V2 - Milos Vasic - 2026-08-21 (rev)</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -456,7 +456,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Two questions about the Simple Flow V2 spec. Each is a plain choice; pick an option and/or type an answer. No technical knowledge needed.</t>
+          <t>Three questions about the Simple Flow V2 spec/tech-plan. Pick an option and/or type an answer. No technical knowledge needed.</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -516,17 +516,17 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>The Jira epic includes an item to rename a column on the Purchase Order page from 'Total Price' to 'Total Cost' (SV-8726). The main Simple Flow V2 spec, in its Purchase Order pages section, does not spell this rename out.</t>
+          <t>The Jira epic includes an item to rename a Purchase Order column from 'Total Price' to 'Total Cost' (SV-8726). The main spec's Purchase Order section does not spell this out.</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Is the 'Total Price' -&gt; 'Total Cost' column rename part of Simple Flow V2, and should our purchase-order test cases check for the label 'Total Cost'?</t>
+          <t>Is that rename part of Simple Flow V2, and should our PO test cases check for 'Total Cost'?</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>A) Yes - it's in scope; test for 'Total Cost'.   B) No - it's separate; leave it out.   C) Something else (please describe).</t>
+          <t>A) Yes - in scope; test for 'Total Cost'.  B) No - separate; leave out.  C) Other.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr"/>
@@ -542,20 +542,46 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>The spec points at a separate ticket (SV-8183) that lists which existing permission each Simple Flow action needs, plus one brand-new permission called 'Received later'. We wrote the permission test cases from that map. That ticket's status in Jira is currently 'Blocked'.</t>
+          <t>The spec points at SV-8183 for which existing permission each action needs, plus a new 'Received later' permission. We wrote the permission cases from it. That ticket's Jira status is 'Blocked'.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Is the permission map in SV-8183 final and safe to test against, or might it still change?</t>
+          <t>Is the SV-8183 permission map final and safe to test against?</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>A) It's final - test against it.   B) It may still change - we'll hold the permission cases until you confirm.   C) Something else (please describe).</t>
+          <t>A) Final - test against it.  B) May change - hold the permission cases.  C) Other.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Simple Flow V2 - when 'Uncomplete' is blocked (Story 19)</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>The spec says a line's 'Uncomplete' action is blocked once the work order is invoiced or paid. The Technical Implementation Plan says that for SERVICE work orders the block actually starts one step earlier, at 'complete'. The two disagree. Our test case follows the spec (invoiced/paid).</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Which is correct for a service work order - is Uncomplete blocked at 'complete', or only at invoiced/paid?</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>A) At 'complete' for service work orders (tech plan) - update the case.  B) At invoiced/paid (spec) - keep as is.  C) Other.</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -568,20 +594,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>QA-ONLY - INTERNAL - NOT FOR MILOS.</t>
+          <t>QA-ONLY - INTERNAL.</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -619,7 +645,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Register id</t>
+          <t>Register</t>
         </is>
       </c>
     </row>
@@ -639,12 +665,12 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Noted rename on PO pages; not separately verified; awaiting scope confirm</t>
+          <t>noted; awaiting scope</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>PO-SF-1 / DD D5</t>
+          <t>PO-SF-1</t>
         </is>
       </c>
     </row>
@@ -654,22 +680,47 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>SV-8183 status Blocked</t>
+          <t>SV-8183 Blocked</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>SFV2-PERM-01..04 + every permissions line</t>
+          <t>SFV2-PERM-01..04</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Authored to SV-8183 map; disclosed ticket is Blocked</t>
+          <t>authored to map; disclosed</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>PO-SF-2 / DD D6</t>
+          <t>PO-SF-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Story 19 tech-plan vs spec (Uncomplete)</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>SFV2-MENU-01</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>kept spec (Rule 57); disclosed (Rule 56)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>PO-SF-3</t>
         </is>
       </c>
     </row>

</xml_diff>